<commit_message>
Added new RDF data schemes and visual schemes for environment-table21-25, and fixed XLSX spreadsheets for environment-table21-25
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table21.xlsx
+++ b/sources/table_normalization/xlsx/environment-table21.xlsx
@@ -404,7 +404,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -505,17 +505,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -526,6 +519,18 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -535,18 +540,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -854,7 +851,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1664,12 +1661,12 @@
       <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="44"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="45"/>
-      <c r="E3" s="45"/>
-      <c r="F3" s="45"/>
-      <c r="G3" s="46" t="s">
+      <c r="B3" s="57"/>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="44" t="s">
         <v>2</v>
       </c>
       <c r="H3" s="7"/>
@@ -1680,23 +1677,23 @@
       <c r="M3" s="7"/>
     </row>
     <row r="4" spans="1:13" ht="26.15" customHeight="1">
-      <c r="A4" s="47" t="s">
+      <c r="A4" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="53" t="s">
+      <c r="B4" s="52"/>
+      <c r="C4" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="56" t="s">
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="56"/>
+      <c r="G4" s="50" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="55.5" customHeight="1">
-      <c r="A5" s="48"/>
-      <c r="B5" s="59" t="s">
+      <c r="A5" s="58"/>
+      <c r="B5" s="53" t="s">
         <v>6</v>
       </c>
       <c r="C5" s="9" t="s">
@@ -1711,7 +1708,7 @@
       <c r="F5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="57"/>
+      <c r="G5" s="51"/>
     </row>
     <row r="6" spans="1:13" ht="24.9" customHeight="1">
       <c r="A6" s="10" t="s">
@@ -2209,7 +2206,7 @@
       </c>
     </row>
     <row r="27" spans="1:16" ht="30" customHeight="1">
-      <c r="A27" s="49" t="s">
+      <c r="A27" s="46" t="s">
         <v>33</v>
       </c>
       <c r="B27" s="32">
@@ -2247,7 +2244,7 @@
       <c r="P27" s="33"/>
     </row>
     <row r="28" spans="1:16" ht="30" customHeight="1">
-      <c r="A28" s="50" t="s">
+      <c r="A28" s="47" t="s">
         <v>34</v>
       </c>
       <c r="B28" s="35">
@@ -2277,7 +2274,7 @@
       <c r="K28" s="36"/>
     </row>
     <row r="29" spans="1:16" ht="30" customHeight="1">
-      <c r="A29" s="50" t="s">
+      <c r="A29" s="47" t="s">
         <v>35</v>
       </c>
       <c r="B29" s="37">
@@ -2307,7 +2304,7 @@
       <c r="K29" s="36"/>
     </row>
     <row r="30" spans="1:16" ht="30" customHeight="1">
-      <c r="A30" s="50" t="s">
+      <c r="A30" s="47" t="s">
         <v>36</v>
       </c>
       <c r="B30" s="38">
@@ -2337,7 +2334,7 @@
       <c r="K30" s="36"/>
     </row>
     <row r="31" spans="1:16" ht="30" customHeight="1">
-      <c r="A31" s="51" t="s">
+      <c r="A31" s="48" t="s">
         <v>37</v>
       </c>
       <c r="B31" s="39">
@@ -2361,7 +2358,7 @@
       <c r="K31" s="36"/>
     </row>
     <row r="32" spans="1:16" ht="17.5">
-      <c r="A32" s="52" t="s">
+      <c r="A32" s="49" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>